<commit_message>
run models, created and updated MS figures
</commit_message>
<xml_diff>
--- a/processed/OSL_Demonstration_Data_Collection_in_Tea_Plantation.xlsx
+++ b/processed/OSL_Demonstration_Data_Collection_in_Tea_Plantation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benjamin\Oath Dropbox\Benjamin Bukombe\tea_paper\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44BE691-5BC7-4423-9859-461B6DED1E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5803AFCD-829C-4EEB-BE45-C9E62ECAF900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,12 +34,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="15">
-  <si>
-    <t>Farm</t>
-  </si>
-  <si>
-    <t>treatment</t>
-  </si>
   <si>
     <t>replicate</t>
   </si>
@@ -78,6 +72,12 @@
   </si>
   <si>
     <t>yield_kg</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Treatment</t>
   </si>
 </sst>
 </file>
@@ -199,8 +199,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:F312">
   <tableColumns count="6">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Farm"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="treatment"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Site"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Treatment"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="area_ha"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="yield_kg"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="replicate"/>
@@ -419,22 +419,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -442,10 +442,10 @@
         <v>46006</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D2" s="3">
         <v>3</v>
@@ -460,10 +460,10 @@
         <v>46006</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" s="3">
         <v>1.5</v>
@@ -478,10 +478,10 @@
         <v>46009</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3">
         <v>2.5000000000000001E-3</v>
@@ -498,10 +498,10 @@
         <v>46009</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="3">
         <v>2.5000000000000001E-3</v>
@@ -518,10 +518,10 @@
         <v>46009</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="3">
         <v>2.5000000000000001E-3</v>
@@ -538,10 +538,10 @@
         <v>46009</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D7" s="3">
         <v>2.5000000000000001E-3</v>
@@ -558,10 +558,10 @@
         <v>46009</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D8" s="3">
         <v>2.5000000000000001E-3</v>
@@ -578,10 +578,10 @@
         <v>46009</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" s="3">
         <v>2.5000000000000001E-3</v>
@@ -598,10 +598,10 @@
         <v>46009</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D10" s="3">
         <v>2.5000000000000001E-3</v>
@@ -618,10 +618,10 @@
         <v>46009</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D11" s="3">
         <v>2.5000000000000001E-3</v>
@@ -638,10 +638,10 @@
         <v>46009</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="3">
         <v>2.5000000000000001E-3</v>
@@ -658,10 +658,10 @@
         <v>46009</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3">
         <v>2.5000000000000001E-3</v>
@@ -678,10 +678,10 @@
         <v>46009</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="3">
         <v>2.5000000000000001E-3</v>
@@ -698,10 +698,10 @@
         <v>46009</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D15" s="3">
         <v>2.5000000000000001E-3</v>
@@ -718,10 +718,10 @@
         <v>46009</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D16" s="3">
         <v>2.5000000000000001E-3</v>
@@ -738,10 +738,10 @@
         <v>46009</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D17" s="3">
         <v>2.5000000000000001E-3</v>
@@ -758,10 +758,10 @@
         <v>46009</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D18" s="3">
         <v>2.5000000000000001E-3</v>
@@ -778,10 +778,10 @@
         <v>46009</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D19" s="3">
         <v>2.5000000000000001E-3</v>
@@ -798,10 +798,10 @@
         <v>46009</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D20" s="3">
         <v>2.5000000000000001E-3</v>
@@ -818,10 +818,10 @@
         <v>46009</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D21" s="3">
         <v>2.5000000000000001E-3</v>
@@ -838,10 +838,10 @@
         <v>46009</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D22" s="3">
         <v>2.5000000000000001E-3</v>
@@ -858,10 +858,10 @@
         <v>46009</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3">
         <v>2.5000000000000001E-3</v>
@@ -878,10 +878,10 @@
         <v>46014</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D24" s="3">
         <v>0.2</v>
@@ -895,10 +895,10 @@
         <v>46014</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D25" s="3">
         <v>0.2</v>
@@ -912,10 +912,10 @@
         <v>46020</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D26" s="3">
         <v>2.5000000000000001E-3</v>
@@ -932,10 +932,10 @@
         <v>46020</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D27" s="3">
         <v>2.5000000000000001E-3</v>
@@ -952,10 +952,10 @@
         <v>46020</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D28" s="3">
         <v>2.5000000000000001E-3</v>
@@ -972,10 +972,10 @@
         <v>46020</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D29" s="3">
         <v>2.5000000000000001E-3</v>
@@ -992,10 +992,10 @@
         <v>46020</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D30" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1012,10 +1012,10 @@
         <v>46020</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D31" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1032,10 +1032,10 @@
         <v>46020</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D32" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1052,10 +1052,10 @@
         <v>46020</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D33" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1072,10 +1072,10 @@
         <v>46020</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D34" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1092,10 +1092,10 @@
         <v>46020</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D35" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1112,10 +1112,10 @@
         <v>46020</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D36" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1132,10 +1132,10 @@
         <v>46020</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D37" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1152,10 +1152,10 @@
         <v>46020</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D38" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1172,10 +1172,10 @@
         <v>46020</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D39" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1192,10 +1192,10 @@
         <v>46020</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D40" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1212,10 +1212,10 @@
         <v>46020</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D41" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1232,10 +1232,10 @@
         <v>46020</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D42" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1252,10 +1252,10 @@
         <v>46020</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D43" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1272,10 +1272,10 @@
         <v>46020</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D44" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1292,10 +1292,10 @@
         <v>46020</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D45" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1312,10 +1312,10 @@
         <v>46021</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D46" s="3">
         <v>3</v>
@@ -1329,10 +1329,10 @@
         <v>46021</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D47" s="3">
         <v>3</v>
@@ -1346,10 +1346,10 @@
         <v>46054</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D48" s="3">
         <v>0.2</v>
@@ -1363,10 +1363,10 @@
         <v>46054</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D49" s="3">
         <v>0.2</v>
@@ -1380,10 +1380,10 @@
         <v>46034</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D50" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1400,10 +1400,10 @@
         <v>46034</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D51" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1420,10 +1420,10 @@
         <v>46034</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D52" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1440,10 +1440,10 @@
         <v>46034</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D53" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1460,10 +1460,10 @@
         <v>46034</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D54" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1480,10 +1480,10 @@
         <v>46034</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D55" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1500,10 +1500,10 @@
         <v>46034</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D56" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1520,10 +1520,10 @@
         <v>46034</v>
       </c>
       <c r="B57" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D57" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1540,10 +1540,10 @@
         <v>46034</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D58" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1560,10 +1560,10 @@
         <v>46034</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D59" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1580,10 +1580,10 @@
         <v>46034</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D60" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1600,10 +1600,10 @@
         <v>46034</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D61" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1620,10 +1620,10 @@
         <v>46034</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D62" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1640,10 +1640,10 @@
         <v>46034</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D63" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1660,10 +1660,10 @@
         <v>46034</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D64" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1680,10 +1680,10 @@
         <v>46034</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D65" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1700,10 +1700,10 @@
         <v>46034</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D66" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1720,10 +1720,10 @@
         <v>46034</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D67" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1740,10 +1740,10 @@
         <v>46034</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D68" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1760,10 +1760,10 @@
         <v>46038</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D69" s="3">
         <v>0.2</v>
@@ -1777,10 +1777,10 @@
         <v>46038</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D70" s="3">
         <v>0.2</v>
@@ -1794,10 +1794,10 @@
         <v>46037</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D71" s="3">
         <v>3</v>
@@ -1811,10 +1811,10 @@
         <v>46037</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D72" s="3">
         <v>3</v>
@@ -1828,10 +1828,10 @@
         <v>46034</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D73" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1848,10 +1848,10 @@
         <v>46048</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D74" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1868,10 +1868,10 @@
         <v>46048</v>
       </c>
       <c r="B75" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D75" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1888,10 +1888,10 @@
         <v>46048</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D76" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1908,10 +1908,10 @@
         <v>46048</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D77" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1928,10 +1928,10 @@
         <v>46048</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D78" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1948,10 +1948,10 @@
         <v>46048</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D79" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1968,10 +1968,10 @@
         <v>46048</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D80" s="3">
         <v>2.5000000000000001E-3</v>
@@ -1988,10 +1988,10 @@
         <v>46048</v>
       </c>
       <c r="B81" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D81" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2008,10 +2008,10 @@
         <v>46048</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D82" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2028,10 +2028,10 @@
         <v>46048</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D83" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2048,10 +2048,10 @@
         <v>46048</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D84" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2068,10 +2068,10 @@
         <v>46048</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D85" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2088,10 +2088,10 @@
         <v>46048</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D86" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2108,10 +2108,10 @@
         <v>46048</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D87" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2128,10 +2128,10 @@
         <v>46048</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D88" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2148,10 +2148,10 @@
         <v>46048</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D89" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2168,10 +2168,10 @@
         <v>46048</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D90" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2188,10 +2188,10 @@
         <v>46048</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D91" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2208,10 +2208,10 @@
         <v>46048</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D92" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2228,10 +2228,10 @@
         <v>46048</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D93" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2248,10 +2248,10 @@
         <v>46050</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D94" s="3">
         <v>0.2</v>
@@ -2265,10 +2265,10 @@
         <v>46050</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D95" s="3">
         <v>0.2</v>
@@ -2282,10 +2282,10 @@
         <v>46051</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D96" s="3">
         <v>3</v>
@@ -2299,10 +2299,10 @@
         <v>46051</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D97" s="3">
         <v>3</v>
@@ -2316,10 +2316,10 @@
         <v>46063</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D98" s="3">
         <v>0.2</v>
@@ -2333,10 +2333,10 @@
         <v>46063</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D99" s="3">
         <v>0.2</v>
@@ -2350,10 +2350,10 @@
         <v>46062</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D100" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2370,10 +2370,10 @@
         <v>46062</v>
       </c>
       <c r="B101" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D101" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2390,10 +2390,10 @@
         <v>46062</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D102" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2410,10 +2410,10 @@
         <v>46062</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D103" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2430,10 +2430,10 @@
         <v>46062</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D104" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2450,10 +2450,10 @@
         <v>46062</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D105" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2470,10 +2470,10 @@
         <v>46062</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D106" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2490,10 +2490,10 @@
         <v>46062</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D107" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2510,10 +2510,10 @@
         <v>46062</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D108" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2530,10 +2530,10 @@
         <v>46062</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D109" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2550,10 +2550,10 @@
         <v>46062</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D110" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2570,10 +2570,10 @@
         <v>46062</v>
       </c>
       <c r="B111" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D111" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2590,10 +2590,10 @@
         <v>46062</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D112" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2610,10 +2610,10 @@
         <v>46062</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D113" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2630,10 +2630,10 @@
         <v>46062</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D114" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2650,10 +2650,10 @@
         <v>46062</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D115" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2670,10 +2670,10 @@
         <v>46062</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D116" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2690,10 +2690,10 @@
         <v>46062</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D117" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2710,10 +2710,10 @@
         <v>46062</v>
       </c>
       <c r="B118" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C118" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D118" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2730,10 +2730,10 @@
         <v>46062</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D119" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2750,10 +2750,10 @@
         <v>46071</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D120" s="3">
         <v>3</v>
@@ -2767,10 +2767,10 @@
         <v>46071</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D121" s="3">
         <v>3</v>
@@ -2784,10 +2784,10 @@
         <v>46077</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D122" s="3">
         <v>0.2</v>
@@ -2801,10 +2801,10 @@
         <v>46077</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D123" s="3">
         <v>0.2</v>
@@ -2818,10 +2818,10 @@
         <v>46078</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D124" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2838,10 +2838,10 @@
         <v>46078</v>
       </c>
       <c r="B125" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D125" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2858,10 +2858,10 @@
         <v>46078</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D126" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2878,10 +2878,10 @@
         <v>46078</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D127" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2898,10 +2898,10 @@
         <v>46078</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D128" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2918,10 +2918,10 @@
         <v>46078</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D129" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2938,10 +2938,10 @@
         <v>46078</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D130" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2958,10 +2958,10 @@
         <v>46078</v>
       </c>
       <c r="B131" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D131" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2978,10 +2978,10 @@
         <v>46078</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D132" s="3">
         <v>2.5000000000000001E-3</v>
@@ -2998,10 +2998,10 @@
         <v>46078</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D133" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3018,10 +3018,10 @@
         <v>46078</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D134" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3038,10 +3038,10 @@
         <v>46078</v>
       </c>
       <c r="B135" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C135" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D135" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3058,10 +3058,10 @@
         <v>46078</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D136" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3078,10 +3078,10 @@
         <v>46078</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D137" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3098,10 +3098,10 @@
         <v>46078</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D138" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3118,10 +3118,10 @@
         <v>46078</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D139" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3138,10 +3138,10 @@
         <v>46078</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D140" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3158,10 +3158,10 @@
         <v>46078</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D141" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3178,10 +3178,10 @@
         <v>46078</v>
       </c>
       <c r="B142" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D142" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3198,10 +3198,10 @@
         <v>46078</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D143" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3218,10 +3218,10 @@
         <v>46083</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D144" s="3">
         <v>3</v>
@@ -3235,10 +3235,10 @@
         <v>46083</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D145" s="3">
         <v>3</v>
@@ -3252,10 +3252,10 @@
         <v>46087</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D146" s="3">
         <v>0.2</v>
@@ -3269,10 +3269,10 @@
         <v>46087</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D147" s="3">
         <v>0.2</v>
@@ -3286,10 +3286,10 @@
         <v>46090</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D148" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3306,10 +3306,10 @@
         <v>46090</v>
       </c>
       <c r="B149" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C149" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C149" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D149" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3326,10 +3326,10 @@
         <v>46090</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D150" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3346,10 +3346,10 @@
         <v>46090</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D151" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3366,10 +3366,10 @@
         <v>46090</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D152" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3386,10 +3386,10 @@
         <v>46090</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D153" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3406,10 +3406,10 @@
         <v>46090</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D154" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3426,10 +3426,10 @@
         <v>46090</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D155" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3446,10 +3446,10 @@
         <v>46090</v>
       </c>
       <c r="B156" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C156" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C156" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D156" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3466,10 +3466,10 @@
         <v>46090</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D157" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3486,10 +3486,10 @@
         <v>46090</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D158" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3506,10 +3506,10 @@
         <v>46090</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D159" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3526,10 +3526,10 @@
         <v>46090</v>
       </c>
       <c r="B160" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C160" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C160" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D160" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3546,10 +3546,10 @@
         <v>46090</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D161" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3566,10 +3566,10 @@
         <v>46090</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D162" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3586,10 +3586,10 @@
         <v>46090</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D163" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3606,10 +3606,10 @@
         <v>46090</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D164" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3626,10 +3626,10 @@
         <v>46090</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D165" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3646,10 +3646,10 @@
         <v>46090</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D166" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3666,10 +3666,10 @@
         <v>46090</v>
       </c>
       <c r="B167" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C167" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C167" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D167" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3686,10 +3686,10 @@
         <v>46090</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D168" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3706,10 +3706,10 @@
         <v>46094</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D169" s="3">
         <v>3</v>
@@ -3723,10 +3723,10 @@
         <v>46094</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D170" s="3">
         <v>3</v>
@@ -3740,10 +3740,10 @@
         <v>46097</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D171" s="3">
         <v>0.2</v>
@@ -3757,10 +3757,10 @@
         <v>46097</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D172" s="3">
         <v>0.2</v>
@@ -3774,10 +3774,10 @@
         <v>46104</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D173" s="3">
         <v>3</v>
@@ -3791,10 +3791,10 @@
         <v>46104</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D174" s="3">
         <v>3</v>
@@ -3808,10 +3808,10 @@
         <v>46106</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D175" s="3">
         <v>0.2</v>
@@ -3825,10 +3825,10 @@
         <v>46106</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D176" s="3">
         <v>0.2</v>
@@ -3842,10 +3842,10 @@
         <v>46114</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D177" s="3">
         <v>3</v>
@@ -3859,10 +3859,10 @@
         <v>46114</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D178" s="3">
         <v>3</v>
@@ -3876,10 +3876,10 @@
         <v>46115</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D179" s="3">
         <v>0.2</v>
@@ -3893,10 +3893,10 @@
         <v>46115</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D180" s="3">
         <v>0.2</v>
@@ -3910,10 +3910,10 @@
         <v>46125</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D181" s="3">
         <v>0.2</v>
@@ -3927,10 +3927,10 @@
         <v>46125</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D182" s="3">
         <v>0.2</v>
@@ -3944,10 +3944,10 @@
         <v>46123</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D183" s="3">
         <v>3</v>
@@ -3961,10 +3961,10 @@
         <v>46123</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D184" s="3">
         <v>3</v>
@@ -3978,10 +3978,10 @@
         <v>46100</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D185" s="3">
         <v>2.5000000000000001E-3</v>
@@ -3998,10 +3998,10 @@
         <v>46100</v>
       </c>
       <c r="B186" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C186" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C186" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D186" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4018,10 +4018,10 @@
         <v>46100</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D187" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4038,10 +4038,10 @@
         <v>46100</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D188" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4058,10 +4058,10 @@
         <v>46100</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D189" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4078,10 +4078,10 @@
         <v>46100</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D190" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4098,10 +4098,10 @@
         <v>46100</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D191" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4118,10 +4118,10 @@
         <v>46100</v>
       </c>
       <c r="B192" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C192" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C192" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D192" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4138,10 +4138,10 @@
         <v>46100</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D193" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4158,10 +4158,10 @@
         <v>46100</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D194" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4178,10 +4178,10 @@
         <v>46100</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D195" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4198,10 +4198,10 @@
         <v>46100</v>
       </c>
       <c r="B196" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C196" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C196" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D196" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4218,10 +4218,10 @@
         <v>46100</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D197" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4238,10 +4238,10 @@
         <v>46100</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D198" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4258,10 +4258,10 @@
         <v>46100</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D199" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4278,10 +4278,10 @@
         <v>46100</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D200" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4298,10 +4298,10 @@
         <v>46100</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D201" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4318,10 +4318,10 @@
         <v>46100</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D202" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4338,10 +4338,10 @@
         <v>46100</v>
       </c>
       <c r="B203" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C203" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C203" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D203" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4358,10 +4358,10 @@
         <v>46100</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D204" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4378,10 +4378,10 @@
         <v>46136</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D205" s="3">
         <v>0.2</v>
@@ -4395,10 +4395,10 @@
         <v>46136</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D206" s="3">
         <v>0.2</v>
@@ -4412,10 +4412,10 @@
         <v>46136</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D207" s="3">
         <v>3</v>
@@ -4429,10 +4429,10 @@
         <v>46136</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D208" s="3">
         <v>3</v>
@@ -4446,10 +4446,10 @@
         <v>46108</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D209" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4466,10 +4466,10 @@
         <v>46108</v>
       </c>
       <c r="B210" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C210" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C210" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D210" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4486,10 +4486,10 @@
         <v>46108</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D211" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4506,10 +4506,10 @@
         <v>46108</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D212" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4526,10 +4526,10 @@
         <v>46108</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D213" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4546,10 +4546,10 @@
         <v>46108</v>
       </c>
       <c r="B214" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D214" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4566,10 +4566,10 @@
         <v>46108</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D215" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4586,10 +4586,10 @@
         <v>46108</v>
       </c>
       <c r="B216" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C216" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C216" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D216" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4606,10 +4606,10 @@
         <v>46108</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D217" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4626,10 +4626,10 @@
         <v>46108</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D218" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4646,10 +4646,10 @@
         <v>46108</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D219" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4666,10 +4666,10 @@
         <v>46108</v>
       </c>
       <c r="B220" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C220" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D220" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4686,10 +4686,10 @@
         <v>46108</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D221" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4706,10 +4706,10 @@
         <v>46108</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C222" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D222" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4726,10 +4726,10 @@
         <v>46108</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D223" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4746,10 +4746,10 @@
         <v>46108</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D224" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4766,10 +4766,10 @@
         <v>46108</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D225" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4786,10 +4786,10 @@
         <v>46108</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C226" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D226" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4806,10 +4806,10 @@
         <v>46108</v>
       </c>
       <c r="B227" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C227" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C227" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D227" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4826,10 +4826,10 @@
         <v>46108</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D228" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4846,10 +4846,10 @@
         <v>46118</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D229" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4866,10 +4866,10 @@
         <v>46118</v>
       </c>
       <c r="B230" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C230" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C230" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D230" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4886,10 +4886,10 @@
         <v>46118</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C231" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D231" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4906,10 +4906,10 @@
         <v>46118</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D232" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4926,10 +4926,10 @@
         <v>46118</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D233" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4946,10 +4946,10 @@
         <v>46118</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D234" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4966,10 +4966,10 @@
         <v>46118</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D235" s="3">
         <v>2.5000000000000001E-3</v>
@@ -4986,10 +4986,10 @@
         <v>46118</v>
       </c>
       <c r="B236" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C236" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C236" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D236" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5006,10 +5006,10 @@
         <v>46118</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D237" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5026,10 +5026,10 @@
         <v>46118</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D238" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5046,10 +5046,10 @@
         <v>46118</v>
       </c>
       <c r="B239" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D239" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5066,10 +5066,10 @@
         <v>46118</v>
       </c>
       <c r="B240" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C240" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C240" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D240" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5086,10 +5086,10 @@
         <v>46118</v>
       </c>
       <c r="B241" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D241" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5106,10 +5106,10 @@
         <v>46118</v>
       </c>
       <c r="B242" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D242" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5126,10 +5126,10 @@
         <v>46118</v>
       </c>
       <c r="B243" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D243" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5146,10 +5146,10 @@
         <v>46118</v>
       </c>
       <c r="B244" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D244" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5166,10 +5166,10 @@
         <v>46118</v>
       </c>
       <c r="B245" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D245" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5186,10 +5186,10 @@
         <v>46118</v>
       </c>
       <c r="B246" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C246" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D246" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5206,10 +5206,10 @@
         <v>46118</v>
       </c>
       <c r="B247" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C247" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C247" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D247" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5226,10 +5226,10 @@
         <v>46118</v>
       </c>
       <c r="B248" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C248" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D248" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5246,10 +5246,10 @@
         <v>46126</v>
       </c>
       <c r="B249" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D249" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5266,10 +5266,10 @@
         <v>46126</v>
       </c>
       <c r="B250" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C250" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C250" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D250" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5286,10 +5286,10 @@
         <v>46126</v>
       </c>
       <c r="B251" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C251" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D251" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5306,10 +5306,10 @@
         <v>46126</v>
       </c>
       <c r="B252" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D252" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5326,10 +5326,10 @@
         <v>46126</v>
       </c>
       <c r="B253" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C253" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D253" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5346,10 +5346,10 @@
         <v>46126</v>
       </c>
       <c r="B254" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D254" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5366,10 +5366,10 @@
         <v>46126</v>
       </c>
       <c r="B255" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C255" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D255" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5386,10 +5386,10 @@
         <v>46126</v>
       </c>
       <c r="B256" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C256" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C256" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D256" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5406,10 +5406,10 @@
         <v>46126</v>
       </c>
       <c r="B257" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D257" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5426,10 +5426,10 @@
         <v>46126</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D258" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5446,10 +5446,10 @@
         <v>46126</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C259" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D259" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5466,10 +5466,10 @@
         <v>46126</v>
       </c>
       <c r="B260" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C260" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C260" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D260" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5486,10 +5486,10 @@
         <v>46126</v>
       </c>
       <c r="B261" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D261" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5506,10 +5506,10 @@
         <v>46126</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C262" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D262" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5526,10 +5526,10 @@
         <v>46126</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C263" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D263" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5546,10 +5546,10 @@
         <v>46126</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C264" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D264" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5566,10 +5566,10 @@
         <v>46126</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C265" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D265" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5586,10 +5586,10 @@
         <v>46126</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D266" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5606,10 +5606,10 @@
         <v>46126</v>
       </c>
       <c r="B267" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C267" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C267" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D267" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5626,10 +5626,10 @@
         <v>46126</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C268" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D268" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5646,10 +5646,10 @@
         <v>46136</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C269" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D269" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5666,10 +5666,10 @@
         <v>46136</v>
       </c>
       <c r="B270" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C270" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C270" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D270" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5686,10 +5686,10 @@
         <v>46136</v>
       </c>
       <c r="B271" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C271" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D271" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5706,10 +5706,10 @@
         <v>46136</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C272" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D272" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5726,10 +5726,10 @@
         <v>46136</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C273" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D273" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5746,10 +5746,10 @@
         <v>46136</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C274" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D274" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5766,10 +5766,10 @@
         <v>46136</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C275" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D275" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5786,10 +5786,10 @@
         <v>46136</v>
       </c>
       <c r="B276" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C276" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C276" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D276" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5806,10 +5806,10 @@
         <v>46136</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C277" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D277" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5826,10 +5826,10 @@
         <v>46136</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C278" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D278" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5846,10 +5846,10 @@
         <v>46136</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C279" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D279" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5866,10 +5866,10 @@
         <v>46136</v>
       </c>
       <c r="B280" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C280" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C280" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D280" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5886,10 +5886,10 @@
         <v>46136</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C281" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D281" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5906,10 +5906,10 @@
         <v>46136</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C282" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D282" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5926,10 +5926,10 @@
         <v>46136</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C283" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D283" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5946,10 +5946,10 @@
         <v>46136</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C284" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D284" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5966,10 +5966,10 @@
         <v>46136</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C285" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D285" s="3">
         <v>2.5000000000000001E-3</v>
@@ -5986,10 +5986,10 @@
         <v>46136</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C286" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D286" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6006,10 +6006,10 @@
         <v>46136</v>
       </c>
       <c r="B287" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C287" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C287" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D287" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6026,10 +6026,10 @@
         <v>46136</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C288" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D288" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6046,10 +6046,10 @@
         <v>46144</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C289" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D289" s="3">
         <v>0.2</v>
@@ -6063,10 +6063,10 @@
         <v>46144</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C290" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D290" s="3">
         <v>0.2</v>
@@ -6080,10 +6080,10 @@
         <v>46146</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C291" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D291" s="3">
         <v>3</v>
@@ -6097,10 +6097,10 @@
         <v>46146</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C292" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D292" s="3">
         <v>3</v>
@@ -6114,10 +6114,10 @@
         <v>46146</v>
       </c>
       <c r="B293" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C293" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D293" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6134,10 +6134,10 @@
         <v>46146</v>
       </c>
       <c r="B294" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C294" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C294" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D294" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6154,10 +6154,10 @@
         <v>46146</v>
       </c>
       <c r="B295" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C295" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D295" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6174,10 +6174,10 @@
         <v>46146</v>
       </c>
       <c r="B296" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C296" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D296" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6194,10 +6194,10 @@
         <v>46146</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C297" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D297" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6214,10 +6214,10 @@
         <v>46146</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C298" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D298" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6234,10 +6234,10 @@
         <v>46146</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C299" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D299" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6254,10 +6254,10 @@
         <v>46146</v>
       </c>
       <c r="B300" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C300" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C300" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D300" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6274,10 +6274,10 @@
         <v>46146</v>
       </c>
       <c r="B301" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C301" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D301" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6294,10 +6294,10 @@
         <v>46146</v>
       </c>
       <c r="B302" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C302" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D302" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6314,10 +6314,10 @@
         <v>46146</v>
       </c>
       <c r="B303" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C303" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D303" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6334,10 +6334,10 @@
         <v>46146</v>
       </c>
       <c r="B304" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C304" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C304" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D304" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6354,10 +6354,10 @@
         <v>46146</v>
       </c>
       <c r="B305" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C305" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D305" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6374,10 +6374,10 @@
         <v>46146</v>
       </c>
       <c r="B306" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C306" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D306" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6394,10 +6394,10 @@
         <v>46146</v>
       </c>
       <c r="B307" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C307" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D307" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6414,10 +6414,10 @@
         <v>46146</v>
       </c>
       <c r="B308" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C308" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D308" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6434,10 +6434,10 @@
         <v>46146</v>
       </c>
       <c r="B309" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C309" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D309" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6454,10 +6454,10 @@
         <v>46146</v>
       </c>
       <c r="B310" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C310" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D310" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6474,10 +6474,10 @@
         <v>46146</v>
       </c>
       <c r="B311" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C311" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C311" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D311" s="3">
         <v>2.5000000000000001E-3</v>
@@ -6494,10 +6494,10 @@
         <v>46146</v>
       </c>
       <c r="B312" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C312" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D312" s="3">
         <v>2.5000000000000001E-3</v>

</xml_diff>